<commit_message>
Atualiza dados da avaliacao 2026
</commit_message>
<xml_diff>
--- a/output/2026/avaliacao_ppgcomp_2026.xlsx
+++ b/output/2026/avaliacao_ppgcomp_2026.xlsx
@@ -4002,7 +4002,7 @@
       </c>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P27" s="2" t="inlineStr">
         <is>
@@ -36999,7 +36999,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L15" s="2" t="n">
         <v>0.25</v>
@@ -45199,7 +45199,7 @@
         <v>0</v>
       </c>
       <c r="K183" s="2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L183" s="2" t="n">
         <v>0.25</v>
@@ -65856,7 +65856,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>365</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">

</xml_diff>